<commit_message>
Phase 2 Complete: Enforced Strict Competence Logic & Purged Non-Mexel Tenders
</commit_message>
<xml_diff>
--- a/01_Tender_Log/Tender_Dashboard_v2.xlsx
+++ b/01_Tender_Log/Tender_Dashboard_v2.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="K14" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Excluded</t>
         </is>
       </c>
       <c r="L14" s="1" t="inlineStr">
@@ -1469,7 +1469,7 @@
         <is>
           <t>High context overlap: power station, plant, treatment
 [Score: 7.2/10 | Priority: HIGH]
-✅ RECOMMENDED - Good opportunity, prepare bid</t>
+✅ RECOMMENDED - Good opportunity, prepare bid [Phase 2: Competence Mismatch]</t>
         </is>
       </c>
       <c r="N14" s="1" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="K15" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Excluded</t>
         </is>
       </c>
       <c r="L15" s="1" t="inlineStr">
@@ -1544,7 +1544,7 @@
         <is>
           <t>Context (power station) + Supporting signal (ro)
 [Score: 8.0/10 | Priority: HIGH]
-🔥 PRIORITY BID - Strong fit, pursue immediately</t>
+🔥 PRIORITY BID - Strong fit, pursue immediately [Phase 2: Competence Mismatch]</t>
         </is>
       </c>
       <c r="N15" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="K16" s="1" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Excluded</t>
         </is>
       </c>
       <c r="L16" s="1" t="inlineStr">
@@ -1619,7 +1619,7 @@
         <is>
           <t>Context (power station) + Supporting signal (ro)
 [Score: 7.2/10 | Priority: HIGH]
-✅ RECOMMENDED - Good opportunity, prepare bid</t>
+✅ RECOMMENDED - Good opportunity, prepare bid [Phase 2: Competence Mismatch]</t>
         </is>
       </c>
       <c r="N16" s="1" t="inlineStr">

</xml_diff>